<commit_message>
BOM changes and added 3d printed parts
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LongRangeEnduranceUAV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E970326-73FE-48F9-9713-6819F386FDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8A6153-534B-449A-A1AD-22C6233BBBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="69">
   <si>
     <t>Item Name</t>
   </si>
@@ -149,9 +149,6 @@
     <t xml:space="preserve">BMS for 4s </t>
   </si>
   <si>
-    <t>Cheap staneless steel wire</t>
-  </si>
-  <si>
     <t>For servo linkages</t>
   </si>
   <si>
@@ -204,6 +201,45 @@
   </si>
   <si>
     <t xml:space="preserve">recycled paper bags in which you buy your grocery, or any kind of packaging paper will do </t>
+  </si>
+  <si>
+    <t>Adhesives</t>
+  </si>
+  <si>
+    <t>CA glue + 2 part epoxy + hotglue</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/male-to-female-jumper-wires-40-pcs-10cm/?gad_source=1&amp;gad_campaignid=17427802559&amp;gclid=EAIaIQobChMIipf1mPmNlQMV05JmAh1UtyQWEAQYASABEgJKCPD_BwE</t>
+  </si>
+  <si>
+    <t>Male to female jumper cables</t>
+  </si>
+  <si>
+    <t>Jumper cables (M-F)</t>
+  </si>
+  <si>
+    <t>Jumper cables (F-F)</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/10cm-female-female-breadboard-jumper-dupont-2-54mm-1p-1p-cable-40-pcs/?gad_source=1&amp;gad_campaignid=17427802559&amp;gclid=EAIaIQobChMIirHDnPmNlQMV_DSDAx3_JBWQEAYYASABEgJp8fD_BwE</t>
+  </si>
+  <si>
+    <t>Female to female jumper cables</t>
+  </si>
+  <si>
+    <t>Cheap stainless steel wire</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/x6b-2-4g-6ch-bus-ppm-pwm-receiver-afhds/</t>
+  </si>
+  <si>
+    <t>Flysky x6b reciever</t>
+  </si>
+  <si>
+    <t>A flysky reciever to land the aircraft once the mission ends</t>
+  </si>
+  <si>
+    <t>Zip Ties, Heat Shrink, Connectors</t>
   </si>
 </sst>
 </file>
@@ -215,7 +251,7 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -268,6 +304,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -296,7 +339,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -311,6 +354,7 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -611,7 +655,7 @@
     </row>
     <row r="5" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -620,7 +664,7 @@
         <v>63.5</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>8</v>
@@ -640,12 +684,12 @@
         <v>16</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -654,10 +698,10 @@
         <v>19.91</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
@@ -770,7 +814,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="2">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D14" t="s">
         <v>35</v>
@@ -781,7 +825,7 @@
     </row>
     <row r="15" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -793,12 +837,12 @@
         <v>16</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -807,15 +851,15 @@
         <v>21.73</v>
       </c>
       <c r="D16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -824,15 +868,15 @@
         <v>4.96</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -844,12 +888,12 @@
         <v>16</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19">
         <v>8</v>
@@ -858,35 +902,94 @@
         <v>0</v>
       </c>
       <c r="D19" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="9" t="s">
+    </row>
+    <row r="20" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="C20" s="12"/>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" s="12">
+        <v>3</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="21" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="4">
-        <v>162.82</v>
-      </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
+      <c r="A21" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0.44</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>59</v>
+      </c>
       <c r="F21" s="6"/>
     </row>
     <row r="22" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="C22" s="2"/>
+      <c r="A22" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" s="2">
+        <v>0.42</v>
+      </c>
+      <c r="D22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="C23" s="2"/>
+      <c r="A23" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" s="2">
+        <v>9.89</v>
+      </c>
+      <c r="D23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="24" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="C24" s="2"/>
+      <c r="A24" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="C25" s="2"/>
@@ -901,6 +1004,12 @@
       <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="4">
+        <v>177.37</v>
+      </c>
       <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">

</xml_diff>